<commit_message>
Normalize image categories to 21-category controlled vocabulary
Fix data-quality issue: 22 distinct raw strings in image_category field
(caused by trailing whitespace and 'Brain TC scan' alias) normalized to
canonical 21-category vocabulary.

Corrections applied:
- 'Endoscopic image ' -> 'Endoscopic image' (trim whitespace)
- 'Brain TC scan' -> 'Brain CT scan' (Italian TC = English CT)

Pipeline validation now enforces image_category vocabulary (check #9).
Shuffled files regenerated with corrected data.
HuggingFace dataset updated with corrected JSON + question_type field.
</commit_message>
<xml_diff>
--- a/Dataset/EN/xlsx/ITAMed_complete_EN.xlsx
+++ b/Dataset/EN/xlsx/ITAMed_complete_EN.xlsx
@@ -40089,7 +40089,7 @@
       </c>
       <c r="M677" t="inlineStr">
         <is>
-          <t>Brain CT Scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="N677" t="inlineStr">
@@ -65955,7 +65955,7 @@
       </c>
       <c r="M1119" t="inlineStr">
         <is>
-          <t>Brain TC scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="N1119" t="inlineStr">

</xml_diff>